<commit_message>
Auto commit 22-06-2025 11:38:53.88
</commit_message>
<xml_diff>
--- a/Templates/MWSS with Compressor Pump.xlsx
+++ b/Templates/MWSS with Compressor Pump.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20325"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Core i5 GAMING\Desktop\estimate-drafter\Templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{760B9C22-515F-4B40-8769-B1AA4645A661}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19420" windowHeight="11020"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19425" windowHeight="11025" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Flushing (Developing) Borewell (Code: GWDDR105)</t>
   </si>
@@ -104,13 +110,31 @@
   </si>
   <si>
     <t>Installation of Single Phase Panel board where new electricity connection is required (Excluding Motor Starter) (Code: GWDDR363)</t>
+  </si>
+  <si>
+    <t>Pump &amp; Accessories</t>
+  </si>
+  <si>
+    <t>Electrification</t>
+  </si>
+  <si>
+    <t>Civil Structures</t>
+  </si>
+  <si>
+    <t>Water Tank &amp; Fittings</t>
+  </si>
+  <si>
+    <t>Supplementory Works</t>
+  </si>
+  <si>
+    <t>Pumping &amp; Distribution Network</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -118,6 +142,14 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -133,7 +165,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -156,11 +188,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -173,6 +231,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -480,22 +544,22 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B36"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="37.81640625" style="4" customWidth="1"/>
-    <col min="2" max="16384" width="9.1796875" style="1"/>
+    <col min="1" max="1" width="37.85546875" style="4" customWidth="1"/>
+    <col min="2" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="29" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -503,87 +567,85 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="29" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="29" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="6"/>
+    </row>
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="58" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="B4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="75" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B5" s="2">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B6" s="2">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B7" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="72.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+    <row r="8" spans="1:2" ht="75" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="29" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="B9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B10" s="2">
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="101.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+    <row r="11" spans="1:2" ht="120" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B11" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="58" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="60" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
@@ -591,7 +653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>12</v>
       </c>
@@ -599,15 +661,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="29" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="58" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="6"/>
+    </row>
+    <row r="15" spans="1:2" ht="60" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>29</v>
       </c>
@@ -615,7 +675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="72.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="75" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
@@ -623,119 +683,168 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="58" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="6"/>
+    </row>
+    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="60" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="101.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="B20" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="6"/>
+    </row>
+    <row r="22" spans="1:2" ht="120" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B22" s="2">
         <v>3000</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="29" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="23" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="29" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="B23" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="B24" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="B25" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="87" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="B26" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27" s="6"/>
+    </row>
+    <row r="28" spans="1:2" ht="105" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B28" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="87" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+    <row r="29" spans="1:2" ht="105" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B29" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="87" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+    <row r="30" spans="1:2" ht="105" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B30" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="87" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+    <row r="31" spans="1:2" ht="105" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B31" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="188.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+    <row r="32" spans="1:2" ht="45" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A33" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="6"/>
+    </row>
+    <row r="34" spans="1:2" ht="210" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B34" s="2">
         <v>250</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="43.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B28" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="87" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+    <row r="35" spans="1:2" ht="105" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B35" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="87" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
+    <row r="36" spans="1:2" ht="90" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B36" s="2">
         <v>6</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A33:B33"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>